<commit_message>
Keep signed adverse slopes; skip Manning velocity when S0 ≤ 0
Ste-Therese profile now shows real signed S0 from survey. Adverse or
flat stations leave y/WSE/V blank instead of using |S0|.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
+++ b/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00000"/>
+  </numFmts>
   <fonts count="6">
     <font>
       <name val="Calibri"/>
@@ -47,7 +49,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +64,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000F5C5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,15 +103,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -472,12 +481,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -500,7 +509,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Q = 7.36 m³/s ; n = 0.035 ; Manning profondeur normale à chaque coupe. Géométrie = sections_stetheres_une_par_une ; pente = Longitudinal.</t>
+          <t>Q = 7.36 m³/s ; n = 0.035 ; Manning profondeur normale si S0 &gt; 0. Pentes adverses: S0 réel affiché, V non calculée (pas de |S0|).</t>
         </is>
       </c>
     </row>
@@ -544,7 +553,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>S0 utilisé</t>
+          <t>S0 réel (signé)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -607,41 +616,27 @@
       <c r="B8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="5" t="n">
-        <v>0.03175</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>0.956</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>35.426</v>
-      </c>
+      <c r="C8" s="6" t="n">
+        <v>-0.03175</v>
+      </c>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
       <c r="F8" s="5" t="n">
         <v>34.47</v>
       </c>
-      <c r="G8" s="5" t="n">
-        <v>2.444</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>5.37</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>0.455</v>
-      </c>
-      <c r="J8" s="6" t="n">
-        <v>3.012</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>1.38</v>
-      </c>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>adverse S0=-0.03175 → use |S0| (approx.)</t>
+          <t>S0 réel adverse = -0.03175 — V non calculée</t>
         </is>
       </c>
     </row>
@@ -675,7 +670,7 @@
       <c r="I9" s="5" t="n">
         <v>0.491</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="J9" s="8" t="n">
         <v>2.521</v>
       </c>
       <c r="K9" s="5" t="n">
@@ -688,7 +683,7 @@
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>from long. table</t>
+          <t>S0 réel (table long.)</t>
         </is>
       </c>
     </row>
@@ -701,41 +696,27 @@
       <c r="B10" s="5" t="n">
         <v>23.663</v>
       </c>
-      <c r="C10" s="5" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>1.259</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>35.679</v>
-      </c>
+      <c r="C10" s="6" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
       <c r="F10" s="5" t="n">
         <v>34.42</v>
       </c>
-      <c r="G10" s="5" t="n">
-        <v>6.692</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>9.906000000000001</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>0.41</v>
-      </c>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+      <c r="J10" s="7" t="n"/>
+      <c r="K10" s="7" t="n"/>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>adverse S0=-0.00250 → use |S0| (approx.)</t>
+          <t>S0 réel adverse = -0.00250 — V non calculée</t>
         </is>
       </c>
     </row>
@@ -769,7 +750,7 @@
       <c r="I11" s="5" t="n">
         <v>0.406</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="J11" s="8" t="n">
         <v>2.235</v>
       </c>
       <c r="K11" s="5" t="n">
@@ -782,7 +763,7 @@
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>from long. table</t>
+          <t>S0 réel (table long.)</t>
         </is>
       </c>
     </row>
@@ -816,7 +797,7 @@
       <c r="I12" s="5" t="n">
         <v>0.326</v>
       </c>
-      <c r="J12" s="6" t="n">
+      <c r="J12" s="8" t="n">
         <v>2.404</v>
       </c>
       <c r="K12" s="5" t="n">
@@ -829,7 +810,7 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>from long. table</t>
+          <t>S0 réel (table long.)</t>
         </is>
       </c>
     </row>
@@ -863,7 +844,7 @@
       <c r="I13" s="5" t="n">
         <v>0.383</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="J13" s="8" t="n">
         <v>1.101</v>
       </c>
       <c r="K13" s="5" t="n">
@@ -876,7 +857,7 @@
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>from long. table</t>
+          <t>S0 réel (table long.)</t>
         </is>
       </c>
     </row>
@@ -910,7 +891,7 @@
       <c r="I14" s="5" t="n">
         <v>0.252</v>
       </c>
-      <c r="J14" s="6" t="n">
+      <c r="J14" s="8" t="n">
         <v>1.504</v>
       </c>
       <c r="K14" s="5" t="n">
@@ -923,7 +904,7 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>from long. table</t>
+          <t>S0 réel (table long.)</t>
         </is>
       </c>
     </row>
@@ -957,7 +938,7 @@
       <c r="I15" s="5" t="n">
         <v>0.739</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="J15" s="8" t="n">
         <v>0.977</v>
       </c>
       <c r="K15" s="5" t="n">
@@ -970,7 +951,7 @@
       </c>
       <c r="M15" s="5" t="inlineStr">
         <is>
-          <t>nearest S0 @ 77.94 m</t>
+          <t>S0 réel nearest @ 77.94 m = 0.00175</t>
         </is>
       </c>
     </row>
@@ -978,11 +959,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>V max</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>3.012</v>
+          <t>V max (S0&gt;0 seulement)</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>2.521</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -993,7 +974,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>V min</t>
+          <t>V min (S0&gt;0 seulement)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1008,7 +989,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>y max</t>
+          <t>y max (S0&gt;0 seulement)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1022,7 +1003,7 @@
     </row>
     <row r="20"/>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1038,30 +1019,54 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• S0 issu du profil longitudinal; pentes adverses → |S0| (approx. friction; un vrai remous amont nécessiterait HEC-RAS).</t>
+          <t>• S0 = pente longitudinale RÉELLE signée du survey (adverse reste négative).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• Fr &gt; 1 ≈ régime torrentiel local.</t>
+          <t>• Si S0 ≤ 0 : pas de calcul Manning → y / WSE / V vides. Pas de |S0|.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>• Si S0 &gt; 0 : V = Q / A à la profondeur normale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>• Fr &gt; 1 ≈ régime torrentiel local.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>• CSV nettoyés dans st_therese_data/ pour relecture.</t>
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>• Lignes orange = pente adverse/nulle. Lignes vertes = Manning OK.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A27:H27"/>
     <mergeCell ref="A22:H22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1074,14 +1079,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Méthode</t>
         </is>
@@ -1100,50 +1105,57 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1) Construire A(WSE), P(WSE) sur la polyligne Distance–Elev</t>
+          <t xml:space="preserve">  1) Lire S0 réel (signé) sur le profil longitudinal à la station de la coupe</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  2) S0 depuis Longitudinal (Station cumulées)</t>
+          <t xml:space="preserve">  2) Si S0 ≤ 0 → arrêter : afficher S0 réel, laisser V / y / WSE vides</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3) Chercher WSE tel que (1/n)·A·R^(2/3)·√S0 = Q</t>
+          <t xml:space="preserve">  3) Si S0 &gt; 0 → construire A(WSE), P(WSE) sur la polyligne Distance–Elev</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4) V = Q / A</t>
+          <t xml:space="preserve">  4) Chercher WSE tel que (1/n)·A·R^(2/3)·√S0 = Q</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5) V = Q / A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Q = 7.36 m³/s, n = 0.035</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Correspondance section → station: 1+000@0, 2+000@13.78, 3+000@23.66, 4+000@35.64,</t>
+          <t>Q = 7.36 m³/s, n = 0.035</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>Correspondance section → station: 1+000@0, 2+000@13.78, 3+000@23.66, 4+000@35.64,</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t xml:space="preserve">  5+000@45.84, 6+000@59.44, 7+000@71.97, 8+000@89.36 m</t>
         </is>
@@ -1166,7 +1178,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Profil longitudinal (données fournies)</t>
+          <t>Profil longitudinal (données fournies) — S0 signé tel quel</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1200,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>S0 réel</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
@@ -1209,7 +1221,7 @@
       <c r="C4" s="5" t="n">
         <v>9.763</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="7" t="n">
         <v>-0.03175</v>
       </c>
       <c r="E4" s="5" t="n">
@@ -1285,7 +1297,7 @@
       <c r="C8" s="5" t="n">
         <v>11.978</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="7" t="n">
         <v>-0.0025</v>
       </c>
       <c r="E8" s="5" t="n">
@@ -1323,7 +1335,7 @@
       <c r="C10" s="5" t="n">
         <v>6.26</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="7" t="n">
         <v>-0.01278</v>
       </c>
       <c r="E10" s="5" t="n">

</xml_diff>

<commit_message>
Add live Excel area/perimeter formulas for Ste-Therese sections
Each coupe gets an Aire_* sheet: edit WSE (yellow) to recompute A and P
from the surveyed polyline with the same trapezoid/triangle segment logic
as the Manning engine.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
+++ b/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
@@ -8,8 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Resultats_Q736" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Methode" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Longitudinal" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Formules_Aire" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Methode" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Longitudinal" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Aire_1000" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Aire_2000" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Aire_3000" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Aire_4000" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Aire_5000" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Aire_6000" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Aire_7000" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Aire_8000" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +27,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.00000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +57,16 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F5C5C"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000F5C5C"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="6">
@@ -103,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,7 +135,12 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -481,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M28"/>
+  <dimension ref="A1:M29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1047,21 +1072,29 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• CSV nettoyés dans st_therese_data/ pour relecture.</t>
+          <t>• Voir onglets Formules_Aire et Aire_* : formules Excel live pour A et P.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>• CSV nettoyés dans st_therese_data/ pour relecture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>• Lignes orange = pente adverse/nulle. Lignes vertes = Manning OK.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A29:H29"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A28:H28"/>
@@ -1073,22 +1106,1399 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 6+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>34.984</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>59.435</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.00535</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>39.414</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>38.58</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>19.598</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>34.92</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>31.09</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>34.21</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>32.472</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>34.28</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>33.532</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>34.78</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>LHE</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),0.5*(($B$2-C14)+($B$2-C15))*ABS(B15-B14),IF(($B$2-C14)&gt;0,0.5*($B$2-C14)*ABS((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14),0.5*($B$2-C15)*ABS(B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),SQRT((B15-B14)^2+(C15-C14)^2),IF(($B$2-C14)&gt;0,SQRT(((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14)^2+($B$2-C14)^2),SQRT((B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14)))^2+($B$2-C15)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>36.689</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>34.96</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>LHE</t>
+        </is>
+      </c>
+      <c r="E15" s="5">
+        <f>$B$2-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),0.5*(($B$2-C15)+($B$2-C16))*ABS(B16-B15),IF(($B$2-C15)&gt;0,0.5*($B$2-C15)*ABS((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15),0.5*($B$2-C16)*ABS(B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),SQRT((B16-B15)^2+(C16-C15)^2),IF(($B$2-C15)&gt;0,SQRT(((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15)^2+($B$2-C15)^2),SQRT((B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15)))^2+($B$2-C16)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>42.646</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>36.57</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E16" s="5">
+        <f>$B$2-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),0.5*(($B$2-C16)+($B$2-C17))*ABS(B17-B16),IF(($B$2-C16)&gt;0,0.5*($B$2-C16)*ABS((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16),0.5*($B$2-C17)*ABS(B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),SQRT((B17-B16)^2+(C17-C16)^2),IF(($B$2-C16)&gt;0,SQRT(((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16)^2+($B$2-C16)^2),SQRT((B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16)))^2+($B$2-C17)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>51.106</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>39.77</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>$B$2-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F19" s="16">
+        <f>SUM(F9:F16)</f>
+        <v/>
+      </c>
+      <c r="G19" s="16">
+        <f>SUM(G9:G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>MIN(C9:C17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>B2-B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B23" s="9">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>IF(B24&gt;0,B23/B24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>IF(OR(B6&lt;=0,B23&lt;=0,B4&lt;=0),0,(1/B6)*B23*(B25^(2/3))*SQRT(B4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>V = Q/A (m/s)</t>
+        </is>
+      </c>
+      <c r="B27" s="9">
+        <f>IF(B23&gt;0,B5/B23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>V utilise Q de B5 (débit de projet). Pour la profondeur normale, ajuster WSE jusqu'à Q_manning ≈ Q.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 7+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>34.5206</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>71.973</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.01742</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>39.35</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>34.48</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>23.05</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>33.59</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>34.056</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>36.37</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>34.946</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>40.43</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F16" s="16">
+        <f>SUM(F9:F13)</f>
+        <v/>
+      </c>
+      <c r="G16" s="16">
+        <f>SUM(G9:G13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>MIN(C9:C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>B2-B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B20" s="9">
+        <f>F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B21" s="9">
+        <f>G16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>IF(B21&gt;0,B20/B21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>IF(OR(B6&lt;=0,B20&lt;=0,B4&lt;=0),0,(1/B6)*B20*(B22^(2/3))*SQRT(B4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>V = Q/A (m/s)</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>IF(B20&gt;0,B5/B20,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>V utilise Q de B5 (débit de projet). Pour la profondeur normale, ajuster WSE jusqu'à Q_manning ≈ Q.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 8+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>35.3257</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>89.361</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.00175</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>39.29</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>37.89</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>15.156</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>36.96</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>24.203</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>35.22</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>27.103</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>33.89</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>29.476</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>33.72</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),0.5*(($B$2-C14)+($B$2-C15))*ABS(B15-B14),IF(($B$2-C14)&gt;0,0.5*($B$2-C14)*ABS((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14),0.5*($B$2-C15)*ABS(B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),SQRT((B15-B14)^2+(C15-C14)^2),IF(($B$2-C14)&gt;0,SQRT(((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14)^2+($B$2-C14)^2),SQRT((B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14)))^2+($B$2-C15)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>34.37</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>BLOC</t>
+        </is>
+      </c>
+      <c r="E15" s="5">
+        <f>$B$2-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),0.5*(($B$2-C15)+($B$2-C16))*ABS(B16-B15),IF(($B$2-C15)&gt;0,0.5*($B$2-C15)*ABS((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15),0.5*($B$2-C16)*ABS(B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),SQRT((B16-B15)^2+(C16-C15)^2),IF(($B$2-C15)&gt;0,SQRT(((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15)^2+($B$2-C15)^2),SQRT((B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15)))^2+($B$2-C16)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>30.297</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>35.66</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E16" s="5">
+        <f>$B$2-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),0.5*(($B$2-C16)+($B$2-C17))*ABS(B17-B16),IF(($B$2-C16)&gt;0,0.5*($B$2-C16)*ABS((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16),0.5*($B$2-C17)*ABS(B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),SQRT((B17-B16)^2+(C17-C16)^2),IF(($B$2-C16)&gt;0,SQRT(((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16)^2+($B$2-C16)^2),SQRT((B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16)))^2+($B$2-C17)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>33.235</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>34.54</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>BLOC</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>$B$2-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F19" s="16">
+        <f>SUM(F9:F16)</f>
+        <v/>
+      </c>
+      <c r="G19" s="16">
+        <f>SUM(G9:G16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>MIN(C9:C17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>B2-B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B23" s="9">
+        <f>F19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>IF(B24&gt;0,B23/B24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>IF(OR(B6&lt;=0,B23&lt;=0,B4&lt;=0),0,(1/B6)*B23*(B25^(2/3))*SQRT(B4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>V = Q/A (m/s)</t>
+        </is>
+      </c>
+      <c r="B27" s="9">
+        <f>IF(B23&gt;0,B5/B23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>V utilise Q de B5 (débit de projet). Pour la profondeur normale, ajuster WSE jusqu'à Q_manning ≈ Q.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Méthode</t>
+          <t>Comment l'aire A est calculée (formules Excel actives dans les onglets Aire_*)</t>
         </is>
       </c>
     </row>
@@ -1098,66 +2508,117 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>À chaque section transversale surveyée:</t>
+          <t>Géométrie: chaque coupe = polyligne Distance (x) vs Elev (z) du fichier sections.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  1) Lire S0 réel (signé) sur le profil longitudinal à la station de la coupe</t>
+          <t>On fixe une cote d'eau WSE. Pour chaque segment [i → i+1]:</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2) Si S0 ≤ 0 → arrêter : afficher S0 réel, laisser V / y / WSE vides</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  3) Si S0 &gt; 0 → construire A(WSE), P(WSE) sur la polyligne Distance–Elev</t>
+          <t xml:space="preserve">  d0 = WSE − z_i     d1 = WSE − z_{i+1}</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4) Chercher WSE tel que (1/n)·A·R^(2/3)·√S0 = Q</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5) V = Q / A</t>
+          <t xml:space="preserve">  1) Segment totalement sec (d0≤0 et d1≤0):     Ai = 0 ,  Pi = 0</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2) Segment totalement mouillé (d0≥0 et d1≥0):</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Q = 7.36 m³/s, n = 0.035</t>
+          <t xml:space="preserve">        Ai = ½ · (d0 + d1) · |x_{i+1} − x_i|     (trapèze)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Correspondance section → station: 1+000@0, 2+000@13.78, 3+000@23.66, 4+000@35.64,</t>
+          <t xml:space="preserve">        Pi = √[(x_{i+1}−x_i)² + (z_{i+1}−z_i)²]  (longueur du fond)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  5+000@45.84, 6+000@59.44, 7+000@71.97, 8+000@89.36 m</t>
+          <t xml:space="preserve">  3) Un bout sec / un bout mouillé: intersection avec WSE en xi,</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Ai = ½ · d_wet · |xi − x_wet|            (triangle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Pi = longueur du bout mouillé jusqu'à xi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A = Σ Ai     P = Σ Pi     R = A/P</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Si S0 &gt; 0:  Q_manning = (1/n)·A·R^(2/3)·√S0     V = Q / A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Onglets Aire_1+000 … Aire_8+000: cellule WSE jaune éditable → A et P se recalculent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>La WSE initiale est celle de la profondeur normale (si S0&gt;0), sinon fond+1 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Les résultats Resultats_Q736 restent les valeurs Manning résolues par Python.</t>
         </is>
       </c>
     </row>
@@ -1172,6 +2633,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Méthode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>À chaque section transversale surveyée:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1) Lire S0 réel (signé) sur le profil longitudinal à la station de la coupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2) Si S0 ≤ 0 → arrêter : afficher S0 réel, laisser V / y / WSE vides</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3) Si S0 &gt; 0 → construire A(WSE), P(WSE) sur la polyligne Distance–Elev</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4) Chercher WSE tel que (1/n)·A·R^(2/3)·√S0 = Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5) V = Q / A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Aire mouillée (détail dans Formules_Aire + onglets Aire_*):</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ai = ½(d0+d1)|Δx| si segment mouillé; triangle si partiellement mouillé; 0 si sec</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A = Σ Ai ; P = Σ Pi ; R = A/P</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Q = 7.36 m³/s, n = 0.035</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Correspondance section → station: 1+000@0, 2+000@13.78, 3+000@23.66, 4+000@35.64,</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  5+000@45.84, 6+000@59.44, 7+000@71.97, 8+000@89.36 m</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1482,4 +3060,2629 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 1+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>35.47</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>-0.03175</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>adverse/nulle — Manning non applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>41.31</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>41.33</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>17.43</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>40.92</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>26.86</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>36.55</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>31.63</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>34.47</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),0.5*(($B$2-C14)+($B$2-C15))*ABS(B15-B14),IF(($B$2-C14)&gt;0,0.5*($B$2-C14)*ABS((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14),0.5*($B$2-C15)*ABS(B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),SQRT((B15-B14)^2+(C15-C14)^2),IF(($B$2-C14)&gt;0,SQRT(((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14)^2+($B$2-C14)^2),SQRT((B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14)))^2+($B$2-C15)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>33.084</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>34.93</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E15" s="5">
+        <f>$B$2-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),0.5*(($B$2-C15)+($B$2-C16))*ABS(B16-B15),IF(($B$2-C15)&gt;0,0.5*($B$2-C15)*ABS((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15),0.5*($B$2-C16)*ABS(B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),SQRT((B16-B15)^2+(C16-C15)^2),IF(($B$2-C15)&gt;0,SQRT(((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15)^2+($B$2-C15)^2),SQRT((B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15)))^2+($B$2-C16)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>35.476</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E16" s="5">
+        <f>$B$2-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),0.5*(($B$2-C16)+($B$2-C17))*ABS(B17-B16),IF(($B$2-C16)&gt;0,0.5*($B$2-C16)*ABS((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16),0.5*($B$2-C17)*ABS(B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),SQRT((B17-B16)^2+(C17-C16)^2),IF(($B$2-C16)&gt;0,SQRT(((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16)^2+($B$2-C16)^2),SQRT((B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16)))^2+($B$2-C17)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>37.766</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>$B$2-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),0.5*(($B$2-C17)+($B$2-C18))*ABS(B18-B17),IF(($B$2-C17)&gt;0,0.5*($B$2-C17)*ABS((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17),0.5*($B$2-C18)*ABS(B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))))))</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),SQRT((B18-B17)^2+(C18-C17)^2),IF(($B$2-C17)&gt;0,SQRT(((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17)^2+($B$2-C17)^2),SQRT((B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17)))^2+($B$2-C18)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>40.855</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>37.13</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E18" s="5">
+        <f>$B$2-C18</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>IF(AND(($B$2-C18)&lt;=0,($B$2-C19)&lt;=0),0,IF(AND(($B$2-C18)&gt;=0,($B$2-C19)&gt;=0),0.5*(($B$2-C18)+($B$2-C19))*ABS(B19-B18),IF(($B$2-C18)&gt;0,0.5*($B$2-C18)*ABS((B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))-B18),0.5*($B$2-C19)*ABS(B19-(B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>IF(AND(($B$2-C18)&lt;=0,($B$2-C19)&lt;=0),0,IF(AND(($B$2-C18)&gt;=0,($B$2-C19)&gt;=0),SQRT((B19-B18)^2+(C19-C18)^2),IF(($B$2-C18)&gt;0,SQRT(((B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))-B18)^2+($B$2-C18)^2),SQRT((B19-(B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18)))^2+($B$2-C19)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>43.953</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>BLOC</t>
+        </is>
+      </c>
+      <c r="E19" s="5">
+        <f>$B$2-C19</f>
+        <v/>
+      </c>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F21" s="16">
+        <f>SUM(F9:F18)</f>
+        <v/>
+      </c>
+      <c r="G21" s="16">
+        <f>SUM(G9:G18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>MIN(C9:C19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>B2-B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B25" s="9">
+        <f>F21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B26" s="9">
+        <f>G21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>IF(B26&gt;0,B25/B26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>S0≤0 → pas de Manning / V</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 2+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>35.514</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>13.783</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.02011</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>9.797000000000001</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>15.147</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>34.93</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>TAB</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>16.46</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>34.57</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),0.5*(($B$2-C14)+($B$2-C15))*ABS(B15-B14),IF(($B$2-C14)&gt;0,0.5*($B$2-C14)*ABS((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14),0.5*($B$2-C15)*ABS(B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),SQRT((B15-B14)^2+(C15-C14)^2),IF(($B$2-C14)&gt;0,SQRT(((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14)^2+($B$2-C14)^2),SQRT((B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14)))^2+($B$2-C15)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>17.76</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>TAB</t>
+        </is>
+      </c>
+      <c r="E15" s="5">
+        <f>$B$2-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),0.5*(($B$2-C15)+($B$2-C16))*ABS(B16-B15),IF(($B$2-C15)&gt;0,0.5*($B$2-C15)*ABS((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15),0.5*($B$2-C16)*ABS(B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),SQRT((B16-B15)^2+(C16-C15)^2),IF(($B$2-C15)&gt;0,SQRT(((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15)^2+($B$2-C15)^2),SQRT((B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15)))^2+($B$2-C16)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>21.518</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>36.43</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E16" s="5">
+        <f>$B$2-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),0.5*(($B$2-C16)+($B$2-C17))*ABS(B17-B16),IF(($B$2-C16)&gt;0,0.5*($B$2-C16)*ABS((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16),0.5*($B$2-C17)*ABS(B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),SQRT((B17-B16)^2+(C17-C16)^2),IF(($B$2-C16)&gt;0,SQRT(((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16)^2+($B$2-C16)^2),SQRT((B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16)))^2+($B$2-C17)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>25.675</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>36.64</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>$B$2-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),0.5*(($B$2-C17)+($B$2-C18))*ABS(B18-B17),IF(($B$2-C17)&gt;0,0.5*($B$2-C17)*ABS((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17),0.5*($B$2-C18)*ABS(B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))))))</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),SQRT((B18-B17)^2+(C18-C17)^2),IF(($B$2-C17)&gt;0,SQRT(((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17)^2+($B$2-C17)^2),SQRT((B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17)))^2+($B$2-C18)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>30.665</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>39.69</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>BLOC</t>
+        </is>
+      </c>
+      <c r="E18" s="5">
+        <f>$B$2-C18</f>
+        <v/>
+      </c>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F20" s="16">
+        <f>SUM(F9:F17)</f>
+        <v/>
+      </c>
+      <c r="G20" s="16">
+        <f>SUM(G9:G17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>MIN(C9:C18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>B2-B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B24" s="9">
+        <f>F20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B25" s="9">
+        <f>G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>IF(B25&gt;0,B24/B25,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>IF(OR(B6&lt;=0,B24&lt;=0,B4&lt;=0),0,(1/B6)*B24*(B26^(2/3))*SQRT(B4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>V = Q/A (m/s)</t>
+        </is>
+      </c>
+      <c r="B28" s="9">
+        <f>IF(B24&gt;0,B5/B24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>V utilise Q de B5 (débit de projet). Pour la profondeur normale, ajuster WSE jusqu'à Q_manning ≈ Q.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 3+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>35.42</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>23.663</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>adverse/nulle — Manning non applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>39.84</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>5.187</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>8.771000000000001</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>36.81</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>11.741</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>35.92</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>13.106</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>34.94</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>TAB</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>13.616</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>34.93</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),0.5*(($B$2-C14)+($B$2-C15))*ABS(B15-B14),IF(($B$2-C14)&gt;0,0.5*($B$2-C14)*ABS((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14),0.5*($B$2-C15)*ABS(B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),SQRT((B15-B14)^2+(C15-C14)^2),IF(($B$2-C14)&gt;0,SQRT(((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14)^2+($B$2-C14)^2),SQRT((B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14)))^2+($B$2-C15)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>14.646</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>34.42</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E15" s="5">
+        <f>$B$2-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),0.5*(($B$2-C15)+($B$2-C16))*ABS(B16-B15),IF(($B$2-C15)&gt;0,0.5*($B$2-C15)*ABS((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15),0.5*($B$2-C16)*ABS(B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),SQRT((B16-B15)^2+(C16-C15)^2),IF(($B$2-C15)&gt;0,SQRT(((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15)^2+($B$2-C15)^2),SQRT((B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15)))^2+($B$2-C16)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>16.266</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>34.89</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E16" s="5">
+        <f>$B$2-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),0.5*(($B$2-C16)+($B$2-C17))*ABS(B17-B16),IF(($B$2-C16)&gt;0,0.5*($B$2-C16)*ABS((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16),0.5*($B$2-C17)*ABS(B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),SQRT((B17-B16)^2+(C17-C16)^2),IF(($B$2-C16)&gt;0,SQRT(((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16)^2+($B$2-C16)^2),SQRT((B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16)))^2+($B$2-C17)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>20.406</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>35.05</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>$B$2-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),0.5*(($B$2-C17)+($B$2-C18))*ABS(B18-B17),IF(($B$2-C17)&gt;0,0.5*($B$2-C17)*ABS((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17),0.5*($B$2-C18)*ABS(B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))))))</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),SQRT((B18-B17)^2+(C18-C17)^2),IF(($B$2-C17)&gt;0,SQRT(((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17)^2+($B$2-C17)^2),SQRT((B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17)))^2+($B$2-C18)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>23.631</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>37.16</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E18" s="5">
+        <f>$B$2-C18</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>IF(AND(($B$2-C18)&lt;=0,($B$2-C19)&lt;=0),0,IF(AND(($B$2-C18)&gt;=0,($B$2-C19)&gt;=0),0.5*(($B$2-C18)+($B$2-C19))*ABS(B19-B18),IF(($B$2-C18)&gt;0,0.5*($B$2-C18)*ABS((B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))-B18),0.5*($B$2-C19)*ABS(B19-(B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>IF(AND(($B$2-C18)&lt;=0,($B$2-C19)&lt;=0),0,IF(AND(($B$2-C18)&gt;=0,($B$2-C19)&gt;=0),SQRT((B19-B18)^2+(C19-C18)^2),IF(($B$2-C18)&gt;0,SQRT(((B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))-B18)^2+($B$2-C18)^2),SQRT((B19-(B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18)))^2+($B$2-C19)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>25.653</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>38.39</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E19" s="5">
+        <f>$B$2-C19</f>
+        <v/>
+      </c>
+      <c r="F19" s="5">
+        <f>IF(AND(($B$2-C19)&lt;=0,($B$2-C20)&lt;=0),0,IF(AND(($B$2-C19)&gt;=0,($B$2-C20)&gt;=0),0.5*(($B$2-C19)+($B$2-C20))*ABS(B20-B19),IF(($B$2-C19)&gt;0,0.5*($B$2-C19)*ABS((B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19))-B19),0.5*($B$2-C20)*ABS(B20-(B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19))))))</f>
+        <v/>
+      </c>
+      <c r="G19" s="5">
+        <f>IF(AND(($B$2-C19)&lt;=0,($B$2-C20)&lt;=0),0,IF(AND(($B$2-C19)&gt;=0,($B$2-C20)&gt;=0),SQRT((B20-B19)^2+(C20-C19)^2),IF(($B$2-C19)&gt;0,SQRT(((B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19))-B19)^2+($B$2-C19)^2),SQRT((B20-(B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19)))^2+($B$2-C20)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>27.412</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>39.62</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>BLOC</t>
+        </is>
+      </c>
+      <c r="E20" s="5">
+        <f>$B$2-C20</f>
+        <v/>
+      </c>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F22" s="16">
+        <f>SUM(F9:F19)</f>
+        <v/>
+      </c>
+      <c r="G22" s="16">
+        <f>SUM(G9:G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>MIN(C9:C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>B2-B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B26" s="9">
+        <f>F22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B27" s="9">
+        <f>G22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>IF(B27&gt;0,B26/B27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>S0≤0 → pas de Manning / V</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 4+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>34.9954</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>35.641</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.02032</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>39.53</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>6.395</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>8.019</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>38.22</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>12.369</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>35.8</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>12.964</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>34.74</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>TAB</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>14.846</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>34.45</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),0.5*(($B$2-C14)+($B$2-C15))*ABS(B15-B14),IF(($B$2-C14)&gt;0,0.5*($B$2-C14)*ABS((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14),0.5*($B$2-C15)*ABS(B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),SQRT((B15-B14)^2+(C15-C14)^2),IF(($B$2-C14)&gt;0,SQRT(((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14)^2+($B$2-C14)^2),SQRT((B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14)))^2+($B$2-C15)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>17.093</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>34.43</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E15" s="5">
+        <f>$B$2-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),0.5*(($B$2-C15)+($B$2-C16))*ABS(B16-B15),IF(($B$2-C15)&gt;0,0.5*($B$2-C15)*ABS((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15),0.5*($B$2-C16)*ABS(B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),SQRT((B16-B15)^2+(C16-C15)^2),IF(($B$2-C15)&gt;0,SQRT(((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15)^2+($B$2-C15)^2),SQRT((B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15)))^2+($B$2-C16)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>18.878</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>34.59</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E16" s="5">
+        <f>$B$2-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),0.5*(($B$2-C16)+($B$2-C17))*ABS(B17-B16),IF(($B$2-C16)&gt;0,0.5*($B$2-C16)*ABS((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16),0.5*($B$2-C17)*ABS(B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))))))</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF(AND(($B$2-C16)&lt;=0,($B$2-C17)&lt;=0),0,IF(AND(($B$2-C16)&gt;=0,($B$2-C17)&gt;=0),SQRT((B17-B16)^2+(C17-C16)^2),IF(($B$2-C16)&gt;0,SQRT(((B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16))-B16)^2+($B$2-C16)^2),SQRT((B17-(B16+(($B$2-C16)/(($B$2-C16)-($B$2-C17)))*(B17-B16)))^2+($B$2-C17)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>20.643</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>34.94</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>TAB</t>
+        </is>
+      </c>
+      <c r="E17" s="5">
+        <f>$B$2-C17</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),0.5*(($B$2-C17)+($B$2-C18))*ABS(B18-B17),IF(($B$2-C17)&gt;0,0.5*($B$2-C17)*ABS((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17),0.5*($B$2-C18)*ABS(B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))))))</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>IF(AND(($B$2-C17)&lt;=0,($B$2-C18)&lt;=0),0,IF(AND(($B$2-C17)&gt;=0,($B$2-C18)&gt;=0),SQRT((B18-B17)^2+(C18-C17)^2),IF(($B$2-C17)&gt;0,SQRT(((B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17))-B17)^2+($B$2-C17)^2),SQRT((B18-(B17+(($B$2-C17)/(($B$2-C17)-($B$2-C18)))*(B18-B17)))^2+($B$2-C18)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>21.275</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>35.77</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E18" s="5">
+        <f>$B$2-C18</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>IF(AND(($B$2-C18)&lt;=0,($B$2-C19)&lt;=0),0,IF(AND(($B$2-C18)&gt;=0,($B$2-C19)&gt;=0),0.5*(($B$2-C18)+($B$2-C19))*ABS(B19-B18),IF(($B$2-C18)&gt;0,0.5*($B$2-C18)*ABS((B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))-B18),0.5*($B$2-C19)*ABS(B19-(B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>IF(AND(($B$2-C18)&lt;=0,($B$2-C19)&lt;=0),0,IF(AND(($B$2-C18)&gt;=0,($B$2-C19)&gt;=0),SQRT((B19-B18)^2+(C19-C18)^2),IF(($B$2-C18)&gt;0,SQRT(((B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18))-B18)^2+($B$2-C18)^2),SQRT((B19-(B18+(($B$2-C18)/(($B$2-C18)-($B$2-C19)))*(B19-B18)))^2+($B$2-C19)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>24.672</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E19" s="5">
+        <f>$B$2-C19</f>
+        <v/>
+      </c>
+      <c r="F19" s="5">
+        <f>IF(AND(($B$2-C19)&lt;=0,($B$2-C20)&lt;=0),0,IF(AND(($B$2-C19)&gt;=0,($B$2-C20)&gt;=0),0.5*(($B$2-C19)+($B$2-C20))*ABS(B20-B19),IF(($B$2-C19)&gt;0,0.5*($B$2-C19)*ABS((B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19))-B19),0.5*($B$2-C20)*ABS(B20-(B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19))))))</f>
+        <v/>
+      </c>
+      <c r="G19" s="5">
+        <f>IF(AND(($B$2-C19)&lt;=0,($B$2-C20)&lt;=0),0,IF(AND(($B$2-C19)&gt;=0,($B$2-C20)&gt;=0),SQRT((B20-B19)^2+(C20-C19)^2),IF(($B$2-C19)&gt;0,SQRT(((B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19))-B19)^2+($B$2-C19)^2),SQRT((B20-(B19+(($B$2-C19)/(($B$2-C19)-($B$2-C20)))*(B20-B19)))^2+($B$2-C20)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>26.991</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>39.53</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>CLO</t>
+        </is>
+      </c>
+      <c r="E20" s="5">
+        <f>$B$2-C20</f>
+        <v/>
+      </c>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F22" s="16">
+        <f>SUM(F9:F19)</f>
+        <v/>
+      </c>
+      <c r="G22" s="16">
+        <f>SUM(G9:G19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>MIN(C9:C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>B2-B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B26" s="9">
+        <f>F22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B27" s="9">
+        <f>G22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>IF(B27&gt;0,B26/B27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>IF(OR(B6&lt;=0,B26&lt;=0,B4&lt;=0),0,(1/B6)*B26*(B28^(2/3))*SQRT(B4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>V = Q/A (m/s)</t>
+        </is>
+      </c>
+      <c r="B30" s="9">
+        <f>IF(B26&gt;0,B5/B26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>V utilise Q de B5 (débit de projet). Pour la profondeur normale, ajuster WSE jusqu'à Q_manning ≈ Q.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Section 5+000 — aire / périmètre mouillés (formules Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>WSE (m)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="n">
+        <v>34.8062</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>← éditer (jaune) : A et P se recalculent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Station cum. (m)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>45.838</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>S0 réel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.0315</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Q (m³/s)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>7.36</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>n Manning</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Distance x (m)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Elev z (m)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Desc</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>d=WSE−z</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Ai segment (m²)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Pi segment (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>39.53</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>BOR</t>
+        </is>
+      </c>
+      <c r="E9" s="5">
+        <f>$B$2-C9</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),0.5*(($B$2-C9)+($B$2-C10))*ABS(B10-B9),IF(($B$2-C9)&gt;0,0.5*($B$2-C9)*ABS((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9),0.5*($B$2-C10)*ABS(B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))))))</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>IF(AND(($B$2-C9)&lt;=0,($B$2-C10)&lt;=0),0,IF(AND(($B$2-C9)&gt;=0,($B$2-C10)&gt;=0),SQRT((B10-B9)^2+(C10-C9)^2),IF(($B$2-C9)&gt;0,SQRT(((B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9))-B9)^2+($B$2-C9)^2),SQRT((B10-(B9+(($B$2-C9)/(($B$2-C9)-($B$2-C10)))*(B10-B9)))^2+($B$2-C10)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>10.522</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>TAH</t>
+        </is>
+      </c>
+      <c r="E10" s="5">
+        <f>$B$2-C10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),0.5*(($B$2-C10)+($B$2-C11))*ABS(B11-B10),IF(($B$2-C10)&gt;0,0.5*($B$2-C10)*ABS((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10),0.5*($B$2-C11)*ABS(B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))))))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF(AND(($B$2-C10)&lt;=0,($B$2-C11)&lt;=0),0,IF(AND(($B$2-C10)&gt;=0,($B$2-C11)&gt;=0),SQRT((B11-B10)^2+(C11-C10)^2),IF(($B$2-C10)&gt;0,SQRT(((B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10))-B10)^2+($B$2-C10)^2),SQRT((B11-(B10+(($B$2-C10)/(($B$2-C10)-($B$2-C11)))*(B11-B10)))^2+($B$2-C11)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>17.92</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>34.326</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E11" s="5">
+        <f>$B$2-C11</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),0.5*(($B$2-C11)+($B$2-C12))*ABS(B12-B11),IF(($B$2-C11)&gt;0,0.5*($B$2-C11)*ABS((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11),0.5*($B$2-C12)*ABS(B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))))))</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>IF(AND(($B$2-C11)&lt;=0,($B$2-C12)&lt;=0),0,IF(AND(($B$2-C11)&gt;=0,($B$2-C12)&gt;=0),SQRT((B12-B11)^2+(C12-C11)^2),IF(($B$2-C11)&gt;0,SQRT(((B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11))-B11)^2+($B$2-C11)^2),SQRT((B12-(B11+(($B$2-C11)/(($B$2-C11)-($B$2-C12)))*(B12-B11)))^2+($B$2-C12)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>20.216</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>34.45</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E12" s="5">
+        <f>$B$2-C12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),0.5*(($B$2-C12)+($B$2-C13))*ABS(B13-B12),IF(($B$2-C12)&gt;0,0.5*($B$2-C12)*ABS((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12),0.5*($B$2-C13)*ABS(B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))))))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF(AND(($B$2-C12)&lt;=0,($B$2-C13)&lt;=0),0,IF(AND(($B$2-C12)&gt;=0,($B$2-C13)&gt;=0),SQRT((B13-B12)^2+(C13-C12)^2),IF(($B$2-C12)&gt;0,SQRT(((B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12))-B12)^2+($B$2-C12)^2),SQRT((B13-(B12+(($B$2-C12)/(($B$2-C12)-($B$2-C13)))*(B13-B12)))^2+($B$2-C13)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>34.296</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>FOND</t>
+        </is>
+      </c>
+      <c r="E13" s="5">
+        <f>$B$2-C13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),0.5*(($B$2-C13)+($B$2-C14))*ABS(B14-B13),IF(($B$2-C13)&gt;0,0.5*($B$2-C13)*ABS((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13),0.5*($B$2-C14)*ABS(B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))))))</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>IF(AND(($B$2-C13)&lt;=0,($B$2-C14)&lt;=0),0,IF(AND(($B$2-C13)&gt;=0,($B$2-C14)&gt;=0),SQRT((B14-B13)^2+(C14-C13)^2),IF(($B$2-C13)&gt;0,SQRT(((B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13))-B13)^2+($B$2-C13)^2),SQRT((B14-(B13+(($B$2-C13)/(($B$2-C13)-($B$2-C14)))*(B14-B13)))^2+($B$2-C14)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>34.87</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>LHE</t>
+        </is>
+      </c>
+      <c r="E14" s="5">
+        <f>$B$2-C14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),0.5*(($B$2-C14)+($B$2-C15))*ABS(B15-B14),IF(($B$2-C14)&gt;0,0.5*($B$2-C14)*ABS((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14),0.5*($B$2-C15)*ABS(B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))))))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF(AND(($B$2-C14)&lt;=0,($B$2-C15)&lt;=0),0,IF(AND(($B$2-C14)&gt;=0,($B$2-C15)&gt;=0),SQRT((B15-B14)^2+(C15-C14)^2),IF(($B$2-C14)&gt;0,SQRT(((B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14))-B14)^2+($B$2-C14)^2),SQRT((B15-(B14+(($B$2-C14)/(($B$2-C14)-($B$2-C15)))*(B15-B14)))^2+($B$2-C15)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>30.703</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>36.55</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="E15" s="5">
+        <f>$B$2-C15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),0.5*(($B$2-C15)+($B$2-C16))*ABS(B16-B15),IF(($B$2-C15)&gt;0,0.5*($B$2-C15)*ABS((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15),0.5*($B$2-C16)*ABS(B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))))))</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>IF(AND(($B$2-C15)&lt;=0,($B$2-C16)&lt;=0),0,IF(AND(($B$2-C15)&gt;=0,($B$2-C16)&gt;=0),SQRT((B16-B15)^2+(C16-C15)^2),IF(($B$2-C15)&gt;0,SQRT(((B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15))-B15)^2+($B$2-C15)^2),SQRT((B16-(B15+(($B$2-C15)/(($B$2-C15)-($B$2-C16)))*(B16-B15)))^2+($B$2-C16)^2))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>34.784</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>39.25</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>THA</t>
+        </is>
+      </c>
+      <c r="E16" s="5">
+        <f>$B$2-C16</f>
+        <v/>
+      </c>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>P = Σ Pi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Totaux</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>A = Σ Ai</t>
+        </is>
+      </c>
+      <c r="F18" s="16">
+        <f>SUM(F9:F15)</f>
+        <v/>
+      </c>
+      <c r="G18" s="16">
+        <f>SUM(G9:G15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Fond min (m)</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>MIN(C9:C16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>y = WSE − fond (m)</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>B2-B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>A (m²)</t>
+        </is>
+      </c>
+      <c r="B22" s="9">
+        <f>F18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>P (m)</t>
+        </is>
+      </c>
+      <c r="B23" s="9">
+        <f>G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>R = A/P (m)</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>IF(B23&gt;0,B22/B23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Q_manning (m³/s)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>IF(OR(B6&lt;=0,B22&lt;=0,B4&lt;=0),0,(1/B6)*B22*(B24^(2/3))*SQRT(B4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>V = Q/A (m/s)</t>
+        </is>
+      </c>
+      <c r="B26" s="9">
+        <f>IF(B22&gt;0,B5/B22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>V utilise Q de B5 (débit de projet). Pour la profondeur normale, ajuster WSE jusqu'à Q_manning ≈ Q.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Drop unused Fr and static OK columns from results table
Keep velocity results with a Remarque column only; Fr and Oui/Non
were not verified by spreadsheet formulas and were not needed here.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
+++ b/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
@@ -137,7 +137,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -520,12 +520,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M27"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -533,9 +533,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,7 +546,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Q = 7.36 m³/s ; n = 0.035 ; Manning profondeur normale si S0 &gt; 0. Pentes adverses: S0 réel affiché, V non calculée (pas de |S0|).</t>
+          <t>Q = 7.36 m³/s ; n = 0.035. Profondeur normale (Manning) si S0 &gt; 0 ; sinon V non calculée.</t>
         </is>
       </c>
     </row>
@@ -574,7 +572,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pour recalculer: éditer build_st_therese_velocity.py puis python build_st_therese_velocity.py</t>
+          <t>Feuilles Section_* : modifier Q et n (jaune) pour recalculer.</t>
         </is>
       </c>
     </row>
@@ -587,12 +585,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Station cum. (m)</t>
+          <t>Station (m)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>S0 réel (signé)</t>
+          <t>S0 (-)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -632,17 +630,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Fr</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>OK?</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>Note S0 / capacité</t>
+          <t>Remarque</t>
         </is>
       </c>
     </row>
@@ -667,13 +655,7 @@
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="8" t="n"/>
       <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>S0 ≤ 0 — profondeur normale non applicable</t>
         </is>
@@ -712,15 +694,7 @@
       <c r="J9" s="10" t="n">
         <v>2.521</v>
       </c>
-      <c r="K9" s="5" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>S0 au profil longitudinal</t>
         </is>
@@ -747,13 +721,7 @@
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="8" t="n"/>
       <c r="J10" s="8" t="n"/>
-      <c r="K10" s="8" t="n"/>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>S0 ≤ 0 — profondeur normale non applicable</t>
         </is>
@@ -792,15 +760,7 @@
       <c r="J11" s="10" t="n">
         <v>2.235</v>
       </c>
-      <c r="K11" s="5" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>S0 au profil longitudinal</t>
         </is>
@@ -839,15 +799,7 @@
       <c r="J12" s="10" t="n">
         <v>2.404</v>
       </c>
-      <c r="K12" s="5" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>S0 au profil longitudinal</t>
         </is>
@@ -886,15 +838,7 @@
       <c r="J13" s="10" t="n">
         <v>1.101</v>
       </c>
-      <c r="K13" s="5" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>S0 au profil longitudinal</t>
         </is>
@@ -933,15 +877,7 @@
       <c r="J14" s="10" t="n">
         <v>1.504</v>
       </c>
-      <c r="K14" s="5" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>S0 au profil longitudinal</t>
         </is>
@@ -980,15 +916,7 @@
       <c r="J15" s="10" t="n">
         <v>0.977</v>
       </c>
-      <c r="K15" s="5" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>S0 interpolé / station 77.94 m</t>
         </is>
@@ -1086,16 +1014,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• Orange = pente adverse/nulle ; vert = calcul OK.</t>
+          <t>• Orange = pente adverse/nulle ; vert = V calculée.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="A22:H22"/>

</xml_diff>

<commit_message>
Make Resultats_Q736 live: Q/n drive all Section sheets in Excel
Office users without Python can change yellow Q or n on the summary
sheet; section results and the table update via formulas.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
+++ b/engineering/drainage-design/channel_profile_velocity/SteTherese_Fosse_Vitesse_Q736.xlsx
@@ -37,7 +37,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +77,11 @@
     <font>
       <i val="1"/>
       <color rgb="009A3412"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -133,16 +138,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,7 +158,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -520,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -546,7 +552,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Q = 7.36 m³/s ; n = 0.035. Profondeur normale (Manning) si S0 &gt; 0 ; sinon V non calculée.</t>
+          <t>Valeurs par défaut Q = 7.36 m³/s ; n = 0.035. Modifier Q ou n (jaune) → le tableau et les Section_* se recalculent (pas besoin de Python).</t>
         </is>
       </c>
     </row>
@@ -572,7 +578,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Feuilles Section_* : modifier Q et n (jaune) pour recalculer.</t>
+          <t>← seules entrées à changer au bureau</t>
         </is>
       </c>
     </row>
@@ -673,26 +679,33 @@
       <c r="C9" s="9" t="n">
         <v>0.02011</v>
       </c>
-      <c r="D9" s="6" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>35.514</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>34.57</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>2.92</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="J9" s="10" t="n">
-        <v>2.521</v>
+      <c r="D9" s="6">
+        <f>'Section_2000'!B10</f>
+        <v/>
+      </c>
+      <c r="E9" s="6">
+        <f>'Section_2000'!B9</f>
+        <v/>
+      </c>
+      <c r="F9" s="6">
+        <f>'Section_2000'!B9-'Section_2000'!B10</f>
+        <v/>
+      </c>
+      <c r="G9" s="6">
+        <f>'Section_2000'!B11</f>
+        <v/>
+      </c>
+      <c r="H9" s="6">
+        <f>'Section_2000'!B12</f>
+        <v/>
+      </c>
+      <c r="I9" s="6">
+        <f>'Section_2000'!B13</f>
+        <v/>
+      </c>
+      <c r="J9" s="10">
+        <f>'Section_2000'!B14</f>
+        <v/>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
@@ -739,26 +752,33 @@
       <c r="C11" s="9" t="n">
         <v>0.02032</v>
       </c>
-      <c r="D11" s="6" t="n">
-        <v>0.5649999999999999</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>34.995</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>34.43</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>3.294</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>8.105</v>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>0.406</v>
-      </c>
-      <c r="J11" s="10" t="n">
-        <v>2.235</v>
+      <c r="D11" s="6">
+        <f>'Section_4000'!B10</f>
+        <v/>
+      </c>
+      <c r="E11" s="6">
+        <f>'Section_4000'!B9</f>
+        <v/>
+      </c>
+      <c r="F11" s="6">
+        <f>'Section_4000'!B9-'Section_4000'!B10</f>
+        <v/>
+      </c>
+      <c r="G11" s="6">
+        <f>'Section_4000'!B11</f>
+        <v/>
+      </c>
+      <c r="H11" s="6">
+        <f>'Section_4000'!B12</f>
+        <v/>
+      </c>
+      <c r="I11" s="6">
+        <f>'Section_4000'!B13</f>
+        <v/>
+      </c>
+      <c r="J11" s="10">
+        <f>'Section_4000'!B14</f>
+        <v/>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
@@ -778,26 +798,33 @@
       <c r="C12" s="9" t="n">
         <v>0.0315</v>
       </c>
-      <c r="D12" s="6" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>34.806</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>34.296</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>3.062</v>
-      </c>
-      <c r="H12" s="6" t="n">
-        <v>9.382</v>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>0.326</v>
-      </c>
-      <c r="J12" s="10" t="n">
-        <v>2.404</v>
+      <c r="D12" s="6">
+        <f>'Section_5000'!B10</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
+        <f>'Section_5000'!B9</f>
+        <v/>
+      </c>
+      <c r="F12" s="6">
+        <f>'Section_5000'!B9-'Section_5000'!B10</f>
+        <v/>
+      </c>
+      <c r="G12" s="6">
+        <f>'Section_5000'!B11</f>
+        <v/>
+      </c>
+      <c r="H12" s="6">
+        <f>'Section_5000'!B12</f>
+        <v/>
+      </c>
+      <c r="I12" s="6">
+        <f>'Section_5000'!B13</f>
+        <v/>
+      </c>
+      <c r="J12" s="10">
+        <f>'Section_5000'!B14</f>
+        <v/>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
@@ -817,26 +844,33 @@
       <c r="C13" s="9" t="n">
         <v>0.00535</v>
       </c>
-      <c r="D13" s="6" t="n">
-        <v>0.774</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>34.984</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>34.21</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>6.683</v>
-      </c>
-      <c r="H13" s="6" t="n">
-        <v>17.467</v>
-      </c>
-      <c r="I13" s="6" t="n">
-        <v>0.383</v>
-      </c>
-      <c r="J13" s="10" t="n">
-        <v>1.101</v>
+      <c r="D13" s="6">
+        <f>'Section_6000'!B10</f>
+        <v/>
+      </c>
+      <c r="E13" s="6">
+        <f>'Section_6000'!B9</f>
+        <v/>
+      </c>
+      <c r="F13" s="6">
+        <f>'Section_6000'!B9-'Section_6000'!B10</f>
+        <v/>
+      </c>
+      <c r="G13" s="6">
+        <f>'Section_6000'!B11</f>
+        <v/>
+      </c>
+      <c r="H13" s="6">
+        <f>'Section_6000'!B12</f>
+        <v/>
+      </c>
+      <c r="I13" s="6">
+        <f>'Section_6000'!B13</f>
+        <v/>
+      </c>
+      <c r="J13" s="10">
+        <f>'Section_6000'!B14</f>
+        <v/>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
@@ -856,26 +890,33 @@
       <c r="C14" s="9" t="n">
         <v>0.01742</v>
       </c>
-      <c r="D14" s="6" t="n">
-        <v>0.465</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>34.521</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>34.056</v>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>4.892</v>
-      </c>
-      <c r="H14" s="6" t="n">
-        <v>19.417</v>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>0.252</v>
-      </c>
-      <c r="J14" s="10" t="n">
-        <v>1.504</v>
+      <c r="D14" s="6">
+        <f>'Section_7000'!B10</f>
+        <v/>
+      </c>
+      <c r="E14" s="6">
+        <f>'Section_7000'!B9</f>
+        <v/>
+      </c>
+      <c r="F14" s="6">
+        <f>'Section_7000'!B9-'Section_7000'!B10</f>
+        <v/>
+      </c>
+      <c r="G14" s="6">
+        <f>'Section_7000'!B11</f>
+        <v/>
+      </c>
+      <c r="H14" s="6">
+        <f>'Section_7000'!B12</f>
+        <v/>
+      </c>
+      <c r="I14" s="6">
+        <f>'Section_7000'!B13</f>
+        <v/>
+      </c>
+      <c r="J14" s="10">
+        <f>'Section_7000'!B14</f>
+        <v/>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
@@ -895,26 +936,33 @@
       <c r="C15" s="9" t="n">
         <v>0.00175</v>
       </c>
-      <c r="D15" s="6" t="n">
-        <v>1.606</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>35.326</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>33.72</v>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>7.533</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>10.191</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>0.739</v>
-      </c>
-      <c r="J15" s="10" t="n">
-        <v>0.977</v>
+      <c r="D15" s="6">
+        <f>'Section_8000'!B10</f>
+        <v/>
+      </c>
+      <c r="E15" s="6">
+        <f>'Section_8000'!B9</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>'Section_8000'!B9-'Section_8000'!B10</f>
+        <v/>
+      </c>
+      <c r="G15" s="6">
+        <f>'Section_8000'!B11</f>
+        <v/>
+      </c>
+      <c r="H15" s="6">
+        <f>'Section_8000'!B12</f>
+        <v/>
+      </c>
+      <c r="I15" s="6">
+        <f>'Section_8000'!B13</f>
+        <v/>
+      </c>
+      <c r="J15" s="10">
+        <f>'Section_8000'!B14</f>
+        <v/>
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
@@ -929,8 +977,9 @@
           <t>V max</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
-        <v>2.521</v>
+      <c r="B17" s="11">
+        <f>MAX(J8:J15)</f>
+        <v/>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -944,8 +993,9 @@
           <t>V min</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
-        <v>0.977</v>
+      <c r="B18" s="12">
+        <f>MIN(J8:J15)</f>
+        <v/>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -959,8 +1009,9 @@
           <t>y max</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
-        <v>1.606</v>
+      <c r="B19" s="12">
+        <f>MAX(D8:D15)</f>
+        <v/>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -979,51 +1030,59 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>• Géométrie : coupes Distance–Élévation du levé.</t>
+          <t>• Modifier Q (B4) ou n (B5) : le tableau se recalcule automatiquement (Excel).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>• S0 issu du profil longitudinal (valeur signée).</t>
+          <t>• Géométrie : coupes Distance–Élévation du levé.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>• S0 ≤ 0 : profondeur normale non applicable (V non calculée).</t>
+          <t>• S0 issu du profil longitudinal (valeur signée).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>• S0 &gt; 0 : Manning, V = Q/A à la profondeur normale.</t>
+          <t>• S0 ≤ 0 : profondeur normale non applicable (V non calculée).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>• Détail par coupe : onglets Section_* ; hypothèses : Notes_calcul.</t>
+          <t>• S0 &gt; 0 : Manning, V = Q/A à la profondeur normale.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>• Détail par coupe : onglets Section_* ; hypothèses : Notes_calcul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>• Orange = pente adverse/nulle ; vert = V calculée.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A28:H28"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="A22:H22"/>
@@ -2122,7 +2181,7 @@
           <t>S0 (-)</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.0315</v>
       </c>
     </row>
@@ -2132,8 +2191,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -2142,8 +2207,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -3442,7 +3513,7 @@
           <t>S0 (-)</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.00535</v>
       </c>
     </row>
@@ -3452,8 +3523,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -3462,8 +3539,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -4786,7 +4869,7 @@
           <t>S0 (-)</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.01742</v>
       </c>
     </row>
@@ -4796,8 +4879,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -4806,8 +4895,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -6058,7 +6153,7 @@
           <t>S0 (-)</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.00175</v>
       </c>
     </row>
@@ -6068,8 +6163,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -6078,8 +6179,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -7370,7 +7477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -7499,7 +7606,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Entrées (jaune) sur chaque feuille Section_* : débit Q et coefficient n.</t>
+          <t>Entrées (jaune) : Q et n sur la feuille Resultats_Q736 uniquement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Modifier Q ou n → toutes les feuilles Section_* et le tableau récapitulatif se mettent à jour.</t>
         </is>
       </c>
     </row>
@@ -7979,8 +8093,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -7989,8 +8109,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -8006,7 +8132,7 @@
           <t>Cote d'eau WSE (m)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
+      <c r="B9" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8014,7 +8140,7 @@
           <t>Profondeur y (m)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
+      <c r="B10" s="20" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8022,7 +8148,7 @@
           <t>Aire A (m²)</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n"/>
+      <c r="B11" s="20" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8030,7 +8156,7 @@
           <t>Périmètre P (m)</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n"/>
+      <c r="B12" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8038,7 +8164,7 @@
           <t>Rayon R = A/P (m)</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n"/>
+      <c r="B13" s="20" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8046,7 +8172,7 @@
           <t>Vitesse V (m/s)</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
+      <c r="B14" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -8299,7 +8425,7 @@
           <t>S0 (-)</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.02011</v>
       </c>
     </row>
@@ -8309,8 +8435,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -8319,8 +8451,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -9682,8 +9820,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -9692,8 +9836,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -9709,7 +9859,7 @@
           <t>Cote d'eau WSE (m)</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n"/>
+      <c r="B9" s="20" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9717,7 +9867,7 @@
           <t>Profondeur y (m)</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n"/>
+      <c r="B10" s="20" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9725,7 +9875,7 @@
           <t>Aire A (m²)</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n"/>
+      <c r="B11" s="20" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9733,7 +9883,7 @@
           <t>Périmètre P (m)</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n"/>
+      <c r="B12" s="20" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9741,7 +9891,7 @@
           <t>Rayon R = A/P (m)</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n"/>
+      <c r="B13" s="20" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9749,7 +9899,7 @@
           <t>Vitesse V (m/s)</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
+      <c r="B14" s="20" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
@@ -10018,7 +10168,7 @@
           <t>S0 (-)</t>
         </is>
       </c>
-      <c r="B4" s="20" t="n">
+      <c r="B4" s="21" t="n">
         <v>0.02032</v>
       </c>
     </row>
@@ -10028,8 +10178,14 @@
           <t>Q (m³/s)</t>
         </is>
       </c>
-      <c r="B5" s="19" t="n">
-        <v>7.36</v>
+      <c r="B5" s="6">
+        <f>'Resultats_Q736'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -10038,8 +10194,14 @@
           <t>n Manning</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>0.035</v>
+      <c r="B6" s="6">
+        <f>'Resultats_Q736'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>lié à Resultats_Q736</t>
+        </is>
       </c>
     </row>
     <row r="8">

</xml_diff>